<commit_message>
[I089] fix(rtm): corrigir referencias aos documentos considerados
Corrige as celulas D7 (Documento de Especificacao de Requisitos:
m2-especificacao-requisitos-v02.md -> m2-especificacao-requisitos-v01.md)
e D8 (Checklist de Aprovacao dos Requisitos:
m2-checklist-aprovacao-requisitos-v01.xlsx ->
m2-checklist-aprovacao-requisitos-v02.xlsx), que citavam um ficheiro
inexistente e uma versao ja substituida.

As 136 linhas da matriz (titulos incluidos) nao foram alteradas.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m2-requirements-traceability-matrix-v01.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m2-requirements-traceability-matrix-v01.xlsx
@@ -867,7 +867,7 @@
       <c r="C7" s="27" t="n"/>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>m2-especificacao-requisitos-v02.md</t>
+          <t>m2-especificacao-requisitos-v01.md</t>
         </is>
       </c>
       <c r="E7" s="28" t="n"/>
@@ -889,7 +889,7 @@
       <c r="C8" s="27" t="n"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>m2-checklist-aprovacao-requisitos-v01.xlsx</t>
+          <t>m2-checklist-aprovacao-requisitos-v02.xlsx</t>
         </is>
       </c>
       <c r="E8" s="28" t="n"/>

</xml_diff>